<commit_message>
Simplify card mappings to permanent employee ownership
</commit_message>
<xml_diff>
--- a/public/templates/card-mappings-template.xlsx
+++ b/public/templates/card-mappings-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Card mappings" sheetId="1" r:id="R0b6babde3c1b4365"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="R1d7df39ead21438b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Card mappings" sheetId="1" r:id="Re529c9577eec424f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" r:id="Rd5097f0ac9124275"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -299,8 +299,8 @@
     <x:col min="2" max="2" width="17.5" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="30.6299991607666" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16.8799991607666" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18.75" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="28.1299991607666" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="35" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="37.5" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -318,284 +318,282 @@
         <x:v>Card user</x:v>
       </x:c>
       <x:c r="E1" s="3" t="str">
-        <x:v>Effective from</x:v>
+        <x:v>ST Person ID</x:v>
       </x:c>
       <x:c r="F1" s="3" t="str">
-        <x:v>Effective through</x:v>
-      </x:c>
-      <x:c r="G1" s="3" t="str">
         <x:v>Reason</x:v>
       </x:c>
+      <x:c r="G1"/>
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="6"/>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
       <x:c r="D2" s="6"/>
-      <x:c r="E2" s="7"/>
-      <x:c r="F2" s="7"/>
-      <x:c r="G2" s="6"/>
+      <x:c r="E2" s="6"/>
+      <x:c r="F2" s="6"/>
+      <x:c r="G2"/>
     </x:row>
     <x:row r="3" ht="27" customHeight="1">
       <x:c r="A3" s="4"/>
       <x:c r="B3" s="4"/>
       <x:c r="C3" s="4"/>
       <x:c r="D3" s="4"/>
-      <x:c r="E3" s="5"/>
-      <x:c r="F3" s="5"/>
-      <x:c r="G3" s="4"/>
+      <x:c r="E3" s="4"/>
+      <x:c r="F3" s="4"/>
+      <x:c r="G3"/>
     </x:row>
     <x:row r="4" ht="27" customHeight="1">
       <x:c r="A4" s="6"/>
       <x:c r="B4" s="6"/>
       <x:c r="C4" s="6"/>
       <x:c r="D4" s="6"/>
-      <x:c r="E4" s="7"/>
-      <x:c r="F4" s="7"/>
-      <x:c r="G4" s="6"/>
+      <x:c r="E4" s="6"/>
+      <x:c r="F4" s="6"/>
+      <x:c r="G4"/>
     </x:row>
     <x:row r="5" ht="27" customHeight="1">
       <x:c r="A5" s="4"/>
       <x:c r="B5" s="4"/>
       <x:c r="C5" s="4"/>
       <x:c r="D5" s="4"/>
-      <x:c r="E5" s="5"/>
-      <x:c r="F5" s="5"/>
-      <x:c r="G5" s="4"/>
+      <x:c r="E5" s="4"/>
+      <x:c r="F5" s="4"/>
+      <x:c r="G5"/>
     </x:row>
     <x:row r="6" ht="27" customHeight="1">
       <x:c r="A6" s="6"/>
       <x:c r="B6" s="6"/>
       <x:c r="C6" s="6"/>
       <x:c r="D6" s="6"/>
-      <x:c r="E6" s="7"/>
-      <x:c r="F6" s="7"/>
-      <x:c r="G6" s="6"/>
+      <x:c r="E6" s="6"/>
+      <x:c r="F6" s="6"/>
+      <x:c r="G6"/>
     </x:row>
     <x:row r="7" ht="27" customHeight="1">
       <x:c r="A7" s="4"/>
       <x:c r="B7" s="4"/>
       <x:c r="C7" s="4"/>
       <x:c r="D7" s="4"/>
-      <x:c r="E7" s="5"/>
-      <x:c r="F7" s="5"/>
-      <x:c r="G7" s="4"/>
+      <x:c r="E7" s="4"/>
+      <x:c r="F7" s="4"/>
+      <x:c r="G7"/>
     </x:row>
     <x:row r="8" ht="27" customHeight="1">
       <x:c r="A8" s="6"/>
       <x:c r="B8" s="6"/>
       <x:c r="C8" s="6"/>
       <x:c r="D8" s="6"/>
-      <x:c r="E8" s="7"/>
-      <x:c r="F8" s="7"/>
-      <x:c r="G8" s="6"/>
+      <x:c r="E8" s="6"/>
+      <x:c r="F8" s="6"/>
+      <x:c r="G8"/>
     </x:row>
     <x:row r="9" ht="27" customHeight="1">
       <x:c r="A9" s="4"/>
       <x:c r="B9" s="4"/>
       <x:c r="C9" s="4"/>
       <x:c r="D9" s="4"/>
-      <x:c r="E9" s="5"/>
-      <x:c r="F9" s="5"/>
-      <x:c r="G9" s="4"/>
+      <x:c r="E9" s="4"/>
+      <x:c r="F9" s="4"/>
+      <x:c r="G9"/>
     </x:row>
     <x:row r="10" ht="27" customHeight="1">
       <x:c r="A10" s="6"/>
       <x:c r="B10" s="6"/>
       <x:c r="C10" s="6"/>
       <x:c r="D10" s="6"/>
-      <x:c r="E10" s="7"/>
-      <x:c r="F10" s="7"/>
-      <x:c r="G10" s="6"/>
+      <x:c r="E10" s="6"/>
+      <x:c r="F10" s="6"/>
+      <x:c r="G10"/>
     </x:row>
     <x:row r="11" ht="27" customHeight="1">
       <x:c r="A11" s="4"/>
       <x:c r="B11" s="4"/>
       <x:c r="C11" s="4"/>
       <x:c r="D11" s="4"/>
-      <x:c r="E11" s="5"/>
-      <x:c r="F11" s="5"/>
-      <x:c r="G11" s="4"/>
+      <x:c r="E11" s="4"/>
+      <x:c r="F11" s="4"/>
+      <x:c r="G11"/>
     </x:row>
     <x:row r="12" ht="27" customHeight="1">
       <x:c r="A12" s="6"/>
       <x:c r="B12" s="6"/>
       <x:c r="C12" s="6"/>
       <x:c r="D12" s="6"/>
-      <x:c r="E12" s="7"/>
-      <x:c r="F12" s="7"/>
-      <x:c r="G12" s="6"/>
+      <x:c r="E12" s="6"/>
+      <x:c r="F12" s="6"/>
+      <x:c r="G12"/>
     </x:row>
     <x:row r="13" ht="27" customHeight="1">
       <x:c r="A13" s="4"/>
       <x:c r="B13" s="4"/>
       <x:c r="C13" s="4"/>
       <x:c r="D13" s="4"/>
-      <x:c r="E13" s="5"/>
-      <x:c r="F13" s="5"/>
-      <x:c r="G13" s="4"/>
+      <x:c r="E13" s="4"/>
+      <x:c r="F13" s="4"/>
+      <x:c r="G13"/>
     </x:row>
     <x:row r="14" ht="27" customHeight="1">
       <x:c r="A14" s="6"/>
       <x:c r="B14" s="6"/>
       <x:c r="C14" s="6"/>
       <x:c r="D14" s="6"/>
-      <x:c r="E14" s="7"/>
-      <x:c r="F14" s="7"/>
-      <x:c r="G14" s="6"/>
+      <x:c r="E14" s="6"/>
+      <x:c r="F14" s="6"/>
+      <x:c r="G14"/>
     </x:row>
     <x:row r="15" ht="27" customHeight="1">
       <x:c r="A15" s="4"/>
       <x:c r="B15" s="4"/>
       <x:c r="C15" s="4"/>
       <x:c r="D15" s="4"/>
-      <x:c r="E15" s="5"/>
-      <x:c r="F15" s="5"/>
-      <x:c r="G15" s="4"/>
+      <x:c r="E15" s="4"/>
+      <x:c r="F15" s="4"/>
+      <x:c r="G15"/>
     </x:row>
     <x:row r="16" ht="27" customHeight="1">
       <x:c r="A16" s="6"/>
       <x:c r="B16" s="6"/>
       <x:c r="C16" s="6"/>
       <x:c r="D16" s="6"/>
-      <x:c r="E16" s="7"/>
-      <x:c r="F16" s="7"/>
-      <x:c r="G16" s="6"/>
+      <x:c r="E16" s="6"/>
+      <x:c r="F16" s="6"/>
+      <x:c r="G16"/>
     </x:row>
     <x:row r="17" ht="27" customHeight="1">
       <x:c r="A17" s="4"/>
       <x:c r="B17" s="4"/>
       <x:c r="C17" s="4"/>
       <x:c r="D17" s="4"/>
-      <x:c r="E17" s="5"/>
-      <x:c r="F17" s="5"/>
-      <x:c r="G17" s="4"/>
+      <x:c r="E17" s="4"/>
+      <x:c r="F17" s="4"/>
+      <x:c r="G17"/>
     </x:row>
     <x:row r="18" ht="27" customHeight="1">
       <x:c r="A18" s="6"/>
       <x:c r="B18" s="6"/>
       <x:c r="C18" s="6"/>
       <x:c r="D18" s="6"/>
-      <x:c r="E18" s="7"/>
-      <x:c r="F18" s="7"/>
-      <x:c r="G18" s="6"/>
+      <x:c r="E18" s="6"/>
+      <x:c r="F18" s="6"/>
+      <x:c r="G18"/>
     </x:row>
     <x:row r="19" ht="27" customHeight="1">
       <x:c r="A19" s="4"/>
       <x:c r="B19" s="4"/>
       <x:c r="C19" s="4"/>
       <x:c r="D19" s="4"/>
-      <x:c r="E19" s="5"/>
-      <x:c r="F19" s="5"/>
-      <x:c r="G19" s="4"/>
+      <x:c r="E19" s="4"/>
+      <x:c r="F19" s="4"/>
+      <x:c r="G19"/>
     </x:row>
     <x:row r="20" ht="27" customHeight="1">
       <x:c r="A20" s="6"/>
       <x:c r="B20" s="6"/>
       <x:c r="C20" s="6"/>
       <x:c r="D20" s="6"/>
-      <x:c r="E20" s="7"/>
-      <x:c r="F20" s="7"/>
-      <x:c r="G20" s="6"/>
+      <x:c r="E20" s="6"/>
+      <x:c r="F20" s="6"/>
+      <x:c r="G20"/>
     </x:row>
     <x:row r="21" ht="27" customHeight="1">
       <x:c r="A21" s="4"/>
       <x:c r="B21" s="4"/>
       <x:c r="C21" s="4"/>
       <x:c r="D21" s="4"/>
-      <x:c r="E21" s="5"/>
-      <x:c r="F21" s="5"/>
-      <x:c r="G21" s="4"/>
+      <x:c r="E21" s="4"/>
+      <x:c r="F21" s="4"/>
+      <x:c r="G21"/>
     </x:row>
     <x:row r="22" ht="27" customHeight="1">
       <x:c r="A22" s="6"/>
       <x:c r="B22" s="6"/>
       <x:c r="C22" s="6"/>
       <x:c r="D22" s="6"/>
-      <x:c r="E22" s="7"/>
-      <x:c r="F22" s="7"/>
-      <x:c r="G22" s="6"/>
+      <x:c r="E22" s="6"/>
+      <x:c r="F22" s="6"/>
+      <x:c r="G22"/>
     </x:row>
     <x:row r="23" ht="27" customHeight="1">
       <x:c r="A23" s="4"/>
       <x:c r="B23" s="4"/>
       <x:c r="C23" s="4"/>
       <x:c r="D23" s="4"/>
-      <x:c r="E23" s="5"/>
-      <x:c r="F23" s="5"/>
-      <x:c r="G23" s="4"/>
+      <x:c r="E23" s="4"/>
+      <x:c r="F23" s="4"/>
+      <x:c r="G23"/>
     </x:row>
     <x:row r="24" ht="27" customHeight="1">
       <x:c r="A24" s="6"/>
       <x:c r="B24" s="6"/>
       <x:c r="C24" s="6"/>
       <x:c r="D24" s="6"/>
-      <x:c r="E24" s="7"/>
-      <x:c r="F24" s="7"/>
-      <x:c r="G24" s="6"/>
+      <x:c r="E24" s="6"/>
+      <x:c r="F24" s="6"/>
+      <x:c r="G24"/>
     </x:row>
     <x:row r="25" ht="27" customHeight="1">
       <x:c r="A25" s="4"/>
       <x:c r="B25" s="4"/>
       <x:c r="C25" s="4"/>
       <x:c r="D25" s="4"/>
-      <x:c r="E25" s="5"/>
-      <x:c r="F25" s="5"/>
-      <x:c r="G25" s="4"/>
+      <x:c r="E25" s="4"/>
+      <x:c r="F25" s="4"/>
+      <x:c r="G25"/>
     </x:row>
     <x:row r="26" ht="27" customHeight="1">
       <x:c r="A26" s="6"/>
       <x:c r="B26" s="6"/>
       <x:c r="C26" s="6"/>
       <x:c r="D26" s="6"/>
-      <x:c r="E26" s="7"/>
-      <x:c r="F26" s="7"/>
-      <x:c r="G26" s="6"/>
+      <x:c r="E26" s="6"/>
+      <x:c r="F26" s="6"/>
+      <x:c r="G26"/>
     </x:row>
     <x:row r="27" ht="27" customHeight="1">
       <x:c r="A27" s="4"/>
       <x:c r="B27" s="4"/>
       <x:c r="C27" s="4"/>
       <x:c r="D27" s="4"/>
-      <x:c r="E27" s="5"/>
-      <x:c r="F27" s="5"/>
-      <x:c r="G27" s="4"/>
+      <x:c r="E27" s="4"/>
+      <x:c r="F27" s="4"/>
+      <x:c r="G27"/>
     </x:row>
     <x:row r="28" ht="27" customHeight="1">
       <x:c r="A28" s="6"/>
       <x:c r="B28" s="6"/>
       <x:c r="C28" s="6"/>
       <x:c r="D28" s="6"/>
-      <x:c r="E28" s="7"/>
-      <x:c r="F28" s="7"/>
-      <x:c r="G28" s="6"/>
+      <x:c r="E28" s="6"/>
+      <x:c r="F28" s="6"/>
+      <x:c r="G28"/>
     </x:row>
     <x:row r="29" ht="27" customHeight="1">
       <x:c r="A29" s="4"/>
       <x:c r="B29" s="4"/>
       <x:c r="C29" s="4"/>
       <x:c r="D29" s="4"/>
-      <x:c r="E29" s="5"/>
-      <x:c r="F29" s="5"/>
-      <x:c r="G29" s="4"/>
+      <x:c r="E29" s="4"/>
+      <x:c r="F29" s="4"/>
+      <x:c r="G29"/>
     </x:row>
     <x:row r="30" ht="27" customHeight="1">
       <x:c r="A30" s="6"/>
       <x:c r="B30" s="6"/>
       <x:c r="C30" s="6"/>
       <x:c r="D30" s="6"/>
-      <x:c r="E30" s="7"/>
-      <x:c r="F30" s="7"/>
-      <x:c r="G30" s="6"/>
+      <x:c r="E30" s="6"/>
+      <x:c r="F30" s="6"/>
+      <x:c r="G30"/>
     </x:row>
     <x:row r="31" ht="27" customHeight="1">
       <x:c r="A31" s="4"/>
       <x:c r="B31" s="4"/>
       <x:c r="C31" s="4"/>
       <x:c r="D31" s="4"/>
-      <x:c r="E31" s="5"/>
-      <x:c r="F31" s="5"/>
-      <x:c r="G31" s="4"/>
+      <x:c r="E31" s="4"/>
+      <x:c r="F31" s="4"/>
+      <x:c r="G31"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -617,7 +615,7 @@
   <x:sheetData>
     <x:row r="1" ht="25" customHeight="1">
       <x:c r="A1" s="8" t="str">
-        <x:v>Richmond | Cardholder mapping uploads</x:v>
+        <x:v>Richmond cardholder mappings</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -659,7 +657,7 @@
     </x:row>
     <x:row r="7" ht="23" customHeight="1">
       <x:c r="A7" s="11" t="str">
-        <x:v>Required: Subaccount ID, Card user, Effective from</x:v>
+        <x:v>Required: Subaccount ID and Card user</x:v>
       </x:c>
       <x:c r="B7" s="10"/>
       <x:c r="C7" s="10"/>
@@ -681,7 +679,7 @@
     </x:row>
     <x:row r="10" ht="23" customHeight="1">
       <x:c r="A10" s="9" t="str">
-        <x:v>Card user is the actual employee who uses the card. Enter dates as YYYY-MM-DD.</x:v>
+        <x:v>Card user is the employee who owns this card. No effective dates are needed.</x:v>
       </x:c>
       <x:c r="B10" s="9"/>
       <x:c r="C10" s="9"/>
@@ -695,7 +693,7 @@
     </x:row>
     <x:row r="12" ht="23" customHeight="1">
       <x:c r="A12" s="11" t="str">
-        <x:v>Optional: Mapping ID, Subaccount name, Effective through, Reason</x:v>
+        <x:v>Optional: Mapping ID, Subaccount name, ST Person ID and Reason</x:v>
       </x:c>
       <x:c r="B12" s="10"/>
       <x:c r="C12" s="10"/>
@@ -717,7 +715,7 @@
     </x:row>
     <x:row r="15" ht="23" customHeight="1">
       <x:c r="A15" s="9" t="str">
-        <x:v>Use Subaccount name as a readable label. Reason records the source of a correction.</x:v>
+        <x:v>Use the ST Person ID from an export to distinguish employees with the same name.</x:v>
       </x:c>
       <x:c r="B15" s="9"/>
       <x:c r="C15" s="9"/>
@@ -739,7 +737,7 @@
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
       <x:c r="A18" s="9" t="str">
-        <x:v>The same subaccount and start date update the existing assignment. Unchanged rows stay unchanged. Cards omitted from the file stay mapped; upload does not delete them.</x:v>
+        <x:v>Each subaccount has one employee mapping for its full purchase history. Repeat uploads correct that mapping and preserve its Mapping ID. Unchanged rows stay unchanged.</x:v>
       </x:c>
       <x:c r="B18" s="9"/>
       <x:c r="C18" s="9"/>
@@ -753,7 +751,7 @@
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
       <x:c r="A20" s="9" t="str">
-        <x:v>A later start date creates a new assignment and ends the earlier open period the day before. A blank end date keeps an existing end date; for a new assignment it means ongoing.</x:v>
+        <x:v>A new employee receives a new card. Omitted and closed cards keep their existing mappings for historical reporting. Uploads never delete mappings.</x:v>
       </x:c>
       <x:c r="B20" s="9"/>
       <x:c r="C20" s="9"/>
@@ -767,7 +765,7 @@
     </x:row>
     <x:row r="22" ht="23" customHeight="1">
       <x:c r="A22" s="9" t="str">
-        <x:v>Retain the Mapping ID when correcting a start date. To reopen an ended assignment, clear its end date in the assignment grid and save the row. Overlapping assignments must be corrected before import.</x:v>
+        <x:v>Use one row per card. Date columns in older templates are ignored. Preview corrections carefully: changing the employee updates all purchases for that card.</x:v>
       </x:c>
       <x:c r="B22" s="9"/>
       <x:c r="C22" s="9"/>

</xml_diff>